<commit_message>
Record final package verification
</commit_message>
<xml_diff>
--- a/docs/gamedev/source-of-truth.xlsx
+++ b/docs/gamedev/source-of-truth.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R57850ab20a274ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R59cb5d843c6f41e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R214ab79f01fd4d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="R52e77caee4d34199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R92207505286f452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="R6c8c557b023f4244"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R1e8cc2be3f224cd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rb73a8114c00c4bd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R97a4730d12da40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5f245973f7054208"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="Rf7f5b0f52d504184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Reb9c954648ef4c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rb779ab4ef68245c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R02091052d2bb4d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Ra4838eedcaf6473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R9a18cd155fe54bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rc272b6e60fb749c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R54c2c46e173c417d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -213,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I8" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I8"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I10" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I10"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K9" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:K9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K12" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:K12"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -635,18 +635,18 @@
         <x:v>Installed Windows/Linux engines, official API, interface, and binding hashes verified</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="7" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A7" s="3" t="str">
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>Local implementation complete; release claim blocked by native macOS and visible-editor gates</x:v>
+        <x:v>Local implementation and deterministic packages complete; release claim blocked by visible editor, controlled performance, native macOS/export, and publication gates</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>Six binaries built/audited; Windows/Linux fixtures pass; GNT-01 to GNT-04 remain fail-closed</x:v>
+        <x:v>Six binaries audited; byte-identical core/demo archives; Windows/Linux archive clean installs and Linux packed runtime pass</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -680,7 +680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a68e12bc8b34936"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d023e49bd604516"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1145,7 +1145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b4c79b57a654003"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07a577af79b43e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2290,7 +2290,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cb30a0bf43148af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade678d22ca94162"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2549,7 +2549,7 @@
         <x:v>docs/gamedev/gauntlet/gnt-03/report.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="8" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A8" s="3" t="str">
         <x:v>MS-055</x:v>
       </x:c>
@@ -2569,7 +2569,7 @@
         <x:v>Platform audits/CI; GNT-04</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Six binaries audited; release gates blocked</x:v>
+        <x:v>Six binaries, deterministic archives, Windows/Linux headless clean installs, and Linux packed runtime complete; release gates blocked</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2581,7 +2581,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bbbb766162849ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ac58d945064d1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2867,10 +2867,68 @@
         <x:v>Native macOS and visible-editor gates remain blocked.</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>BLD-065</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="str">
+        <x:v>Deterministic archives</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="str">
+        <x:v>Packaged clean commit 4e6a8c0 twice and compared complete ZIP bytes.</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="str">
+        <x:v>scripts/package_release.py; final desktop addon roots</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="str">
+        <x:v>4e6a8c0</x:v>
+      </x:c>
+      <x:c r="G9" s="3" t="str">
+        <x:v>Core/demo SHA-256 equality and file-level manifests</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I9" s="3" t="str">
+        <x:v>Core 78 entries; demo 171 entries; both runs byte-identical.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>BLD-075</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>Archive clean install</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>Extracted the final core ZIP and ran Windows/Linux editor and forced-release fixtures plus a new packed Linux PCK.</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>final core ZIP; tests/fixture; scripts/run_fixture.py</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>4e6a8c0</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>Four 11-case runs and one packed 11-case run; zero suspicious lines</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="str">
+        <x:v>Visible authoring and native Windows/macOS exports remain gated.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3d818ed6a5c4c10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f9d45332eaf4e87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3251,10 +3309,115 @@
         <x:v>DominicBytes</x:v>
       </x:c>
     </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>QA-075</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>MS-055</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>Deterministic archive comparison</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>Clean source commit 4e6a8c0; two independent output roots</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>Core and demo ZIP bytes match</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>Core 4BAA0069...F261298 and demo 30456BCF...ECC8A3 match exactly</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>reports/licenses/limboai-package-audit.md</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J10" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="K10" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A11" s="3" t="str">
+        <x:v>QA-085</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="str">
+        <x:v>MS-055</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="str">
+        <x:v>Core archive clean install</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="str">
+        <x:v>Windows host and offline Ubuntu 24.04; editor and template_release</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="str">
+        <x:v>All 11 cases pass with zero suspicious lines</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="str">
+        <x:v>Four profiles pass from a fresh archive extraction</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
+        <x:v>reports/test-results/automated-desktop.md</x:v>
+      </x:c>
+      <x:c r="I11" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J11" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="K11" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A12" s="3" t="str">
+        <x:v>QA-095</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="str">
+        <x:v>MS-055</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="str">
+        <x:v>Packed Linux runtime</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>Exact packaged Linux template_release library; 89-file PCK</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="str">
+        <x:v>All 11 cases pass with zero suspicious lines</x:v>
+      </x:c>
+      <x:c r="G12" s="3" t="str">
+        <x:v>PCK SHA-256 2A200601...EA69DE35; runtime PASS</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str">
+        <x:v>reports/test-results/automated-desktop.md</x:v>
+      </x:c>
+      <x:c r="I12" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J12" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="K12" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41e9a365db5240fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49afa835a9604df6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3635,7 +3798,7 @@
         <x:v>BLOCKERS.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>RSK-009</x:v>
       </x:c>
@@ -3652,7 +3815,7 @@
         <x:v>Addon may be correct but unusable.</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>Four 200-agent smoke samples pass; five-run and visible 100%/150% protocols remain blocked.</x:v>
+        <x:v>Final-build, archive-clean-install, and packed-runtime 200-agent smoke samples pass; controlled five-run and visible 100%/150% protocols remain blocked.</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
         <x:v>Codex</x:v>
@@ -3670,7 +3833,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re856b3851eb34f14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0cdd1bf8174576"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3817,7 +3980,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="3" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="str">
         <x:v>REL-001</x:v>
       </x:c>
@@ -3828,7 +3991,7 @@
         <x:v>1.6.0+redot.26.2.1</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>2e32af7</x:v>
+        <x:v>4e6a8c0</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
         <x:v>Windows x86-64; Linux x86-64; macOS universal</x:v>
@@ -3837,13 +4000,13 @@
         <x:v>Editor + template_release</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Six local native binaries; core/demo ZIPs pending clean double-package run</x:v>
+        <x:v>Core ZIP (78 entries), demo ZIP (171 entries), and six local native binaries</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>See automated-desktop.md</x:v>
+        <x:v>Core 4BAA00697195CF9EFDDC8DE38565D7528ABD5D967FFA04E5BBC4D22E6F261298; Demo 30456BCF232E029368CBB9913F850581356C15A384F5E1CE3E4C0EB417ECC8A3</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Windows/Linux runtime PASS; macOS structural PASS</x:v>
+        <x:v>Double-package MATCH; Windows/Linux archive clean install PASS; Linux packed PCK PASS; macOS structural PASS</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
         <x:v>No publication</x:v>
@@ -3852,13 +4015,13 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L3" s="3" t="str">
-        <x:v>Native macOS, visible editor, export, signing, and owner authorization gates remain.</x:v>
+        <x:v>Native macOS, visible editor, controlled performance, native Windows/macOS export, signing, and owner authorization gates remain.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a42744542794e89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5880e6c896841c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4030,7 +4193,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4572bc1f8b94939"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd776f17b4bca4f12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile final Linux package evidence
</commit_message>
<xml_diff>
--- a/docs/gamedev/source-of-truth.xlsx
+++ b/docs/gamedev/source-of-truth.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R5f245973f7054208"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="Rf7f5b0f52d504184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Reb9c954648ef4c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rb779ab4ef68245c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R02091052d2bb4d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Ra4838eedcaf6473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R9a18cd155fe54bc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rc272b6e60fb749c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R54c2c46e173c417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re0581b0e942342af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R85ac9d06efd74826"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R87d3eb7153f9483b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rf69382e00fc142e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R21a0cd894b634a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Ree0379e798ef413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R6169130b0c0f4142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Re9cac292d3984869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R61baccea8c074256"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -213,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I10" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I11" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I11"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K12" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:K12"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K13" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:K13"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -635,7 +635,7 @@
         <x:v>Installed Windows/Linux engines, official API, interface, and binding hashes verified</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="7" ht="66" hidden="0" customHeight="1">
       <x:c r="A7" s="3" t="str">
         <x:v>Status</x:v>
       </x:c>
@@ -646,7 +646,7 @@
         <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>Six binaries audited; byte-identical core/demo archives; Windows/Linux archive clean installs and Linux packed runtime pass</x:v>
+        <x:v>Six binaries audited; byte-identical core/demo archives; Windows/Linux archive clean installs and Linux packed runtime pass; Ubuntu 24.04/glibc 2.38 floor declared</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -680,7 +680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d023e49bd604516"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6b150f609204fbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1145,7 +1145,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07a577af79b43e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R423b50baed1a45e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2113,10 +2113,10 @@
         <x:v>SConstruct verifies the exact pre-populated binding/API/interface and emits only the desktop matrix.</x:v>
       </x:c>
       <x:c r="M17" s="3" t="str">
-        <x:v>Windows/Linux runtime and all six structural audits pass.</x:v>
+        <x:v>Windows/Linux runtime and all six structural audits pass; Linux GLIBC_2.38 ceiling is enforced.</x:v>
       </x:c>
       <x:c r="N17" s="3" t="str">
-        <x:v>Use external project roots; native macOS CI remains authoritative.</x:v>
+        <x:v>Use external project roots; declare the Ubuntu 24.04/glibc 2.38 floor; native macOS CI remains authoritative.</x:v>
       </x:c>
       <x:c r="O17" s="3" t="str">
         <x:v>SConstruct; deps.env; gdextension/limboai.gdextension</x:v>
@@ -2290,7 +2290,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade678d22ca94162"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9d513f27bc84519"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2581,7 +2581,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ac58d945064d1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e7718a5bb8f4bf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2878,13 +2878,13 @@
         <x:v>Deterministic archives</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>Packaged clean commit 4e6a8c0 twice and compared complete ZIP bytes.</x:v>
+        <x:v>Packaged clean commit f51be6ba twice and compared complete ZIP bytes.</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
         <x:v>scripts/package_release.py; final desktop addon roots</x:v>
       </x:c>
       <x:c r="F9" s="3" t="str">
-        <x:v>4e6a8c0</x:v>
+        <x:v>f51be6ba</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
         <x:v>Core/demo SHA-256 equality and file-level manifests</x:v>
@@ -2913,7 +2913,7 @@
         <x:v>final core ZIP; tests/fixture; scripts/run_fixture.py</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
-        <x:v>4e6a8c0</x:v>
+        <x:v>f51be6ba</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>Four 11-case runs and one packed 11-case run; zero suspicious lines</x:v>
@@ -2923,12 +2923,41 @@
       </x:c>
       <x:c r="I10" s="3" t="str">
         <x:v>Visible authoring and native Windows/macOS exports remain gated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A11" s="3" t="str">
+        <x:v>BLD-085</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="str">
+        <x:v>Linux compatibility floor</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="str">
+        <x:v>Documented and audit-locked the packaged Linux requirement to glibc 2.38 or older at build time.</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="str">
+        <x:v>COMPATIBILITY.md; LIMITATIONS.md; scripts/audit_linux_binary.sh</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="str">
+        <x:v>f51be6ba</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="str">
+        <x:v>Both final ELF libraries report GLIBC_MAX 2.38</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I11" s="3" t="str">
+        <x:v>Provided binaries target Ubuntu 24.04/glibc 2.38+; older distributions require a source rebuild.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f9d45332eaf4e87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red05e9cf6a0c4176"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3323,13 +3352,13 @@
         <x:v>Deterministic archive comparison</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
-        <x:v>Clean source commit 4e6a8c0; two independent output roots</x:v>
+        <x:v>Clean source commit f51be6ba; two independent output roots</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
         <x:v>Core and demo ZIP bytes match</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Core 4BAA0069...F261298 and demo 30456BCF...ECC8A3 match exactly</x:v>
+        <x:v>Core FF4E028C...D1FEE70 and demo 30456BCF...ECC8A3 match exactly</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
         <x:v>reports/licenses/limboai-package-audit.md</x:v>
@@ -3399,7 +3428,7 @@
         <x:v>All 11 cases pass with zero suspicious lines</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>PCK SHA-256 2A200601...EA69DE35; runtime PASS</x:v>
+        <x:v>PCK SHA-256 63F19B07...645AD13CB; runtime PASS</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3411,13 +3440,48 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="3" t="str">
+        <x:v>QA-105</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="str">
+        <x:v>MS-055</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="str">
+        <x:v>Linux glibc version ceiling</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="str">
+        <x:v>Pinned ELF audit against both final Linux libraries</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:v>No required GLIBC symbol version exceeds 2.38</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="str">
+        <x:v>Editor and template_release each report GLIBC_MAX 2.38</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str">
+        <x:v>scripts/audit_linux_binary.sh</x:v>
+      </x:c>
+      <x:c r="I13" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J13" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="K13" s="3" t="str">
         <x:v>Codex</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49afa835a9604df6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dd999123d904150"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3702,7 +3766,7 @@
         <x:v>docs/gamedev/gauntlet/gnt-02/report.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A8" s="3" t="str">
         <x:v>RSK-006</x:v>
       </x:c>
@@ -3719,7 +3783,7 @@
         <x:v>Desktop release could be incomplete.</x:v>
       </x:c>
       <x:c r="F8" s="3" t="str">
-        <x:v>Six structural audits pass; native macOS workflow remains authoritative for runtime.</x:v>
+        <x:v>Six structural audits pass; Linux glibc 2.38 floor is declared and enforced; native macOS workflow remains authoritative for runtime.</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
         <x:v>Codex</x:v>
@@ -3833,7 +3897,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc0cdd1bf8174576"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50b12436eade48d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3991,7 +4055,7 @@
         <x:v>1.6.0+redot.26.2.1</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>4e6a8c0</x:v>
+        <x:v>f51be6ba</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
         <x:v>Windows x86-64; Linux x86-64; macOS universal</x:v>
@@ -4003,7 +4067,7 @@
         <x:v>Core ZIP (78 entries), demo ZIP (171 entries), and six local native binaries</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>Core 4BAA00697195CF9EFDDC8DE38565D7528ABD5D967FFA04E5BBC4D22E6F261298; Demo 30456BCF232E029368CBB9913F850581356C15A384F5E1CE3E4C0EB417ECC8A3</x:v>
+        <x:v>Core FF4E028C09784A1C0F83BBC1F0AB6EAF6D6BB0FBD046F22745F463E94D1FEE70; Demo 30456BCF232E029368CBB9913F850581356C15A384F5E1CE3E4C0EB417ECC8A3</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
         <x:v>Double-package MATCH; Windows/Linux archive clean install PASS; Linux packed PCK PASS; macOS structural PASS</x:v>
@@ -4015,13 +4079,13 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L3" s="3" t="str">
-        <x:v>Native macOS, visible editor, controlled performance, native Windows/macOS export, signing, and owner authorization gates remain.</x:v>
+        <x:v>Linux requires glibc 2.38+; native macOS, visible editor, controlled performance, native Windows/macOS export, signing, and owner authorization gates remain.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5880e6c896841c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62e0d8a08984d60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4193,7 +4257,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd776f17b4bca4f12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57731cb8c4d14210"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Approve LimboAI 1.8 Redot port baseline
</commit_message>
<xml_diff>
--- a/docs/gamedev/source-of-truth.xlsx
+++ b/docs/gamedev/source-of-truth.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re0581b0e942342af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R85ac9d06efd74826"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R87d3eb7153f9483b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rf69382e00fc142e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R21a0cd894b634a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Ree0379e798ef413f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R6169130b0c0f4142"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Re9cac292d3984869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R61baccea8c074256"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R640a302ed2c444e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="Red8624fc5cd44913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R35fa68da42894afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="R1734571317c54430"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R2776dec544584180"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Rf8f1f53615a2437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="Re600bc6666e441bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rf3bb6f2bb0464d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="Rc9cfedd505e04386"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -151,8 +151,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GameDev2" displayName="GameDev2" ref="A1:I14" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GameDev2" displayName="GameDev2" ref="A1:I15" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GameDev3" displayName="GameDev3" ref="A1:Q20" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:Q20"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GameDev3" displayName="GameDev3" ref="A1:Q21" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:Q21"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -213,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I11" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I11"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I12" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I12"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K13" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:K13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K14" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:K14"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -640,13 +640,13 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>Local implementation and deterministic packages complete; release claim blocked by visible editor, controlled performance, native macOS/export, and publication gates</x:v>
+        <x:v>LimboAI v1.8.0 Redot port in progress; the verified 1.6 implementation is retained as a checkpoint and all implementation gates are reopened for the new baseline</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>Six binaries audited; byte-identical core/demo archives; Windows/Linux archive clean installs and Linux packed runtime pass; Ubuntu 24.04/glibc 2.38 floor declared</x:v>
+        <x:v>Owner-authorized scope expansion to the complete v1.8 feature set on Redot 26.2</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -680,7 +680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6b150f609204fbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a3aa6dd9d5742d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -814,7 +814,7 @@
         <x:v>Port v1.8.0; use an unpinned branch</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
         <x:v>Codex</x:v>
@@ -1142,10 +1142,39 @@
         <x:v>BLOCKERS.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="3" t="str">
+        <x:v>DEC-125</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C15" s="3" t="str">
+        <x:v>Baseline and scope</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="str">
+        <x:v>Promote upstream LimboAI v1.8.0 at 3fbd85118b924d50c10a495ad5c7175028649d77 to the Redot port baseline.</x:v>
+      </x:c>
+      <x:c r="E15" s="3" t="str">
+        <x:v>The owner explicitly requires the complete 1.8 feature set and directed that it build on the verified 1.6 Redot compatibility foundation.</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="str">
+        <x:v>Remain on v1.6.0; selectively backport more features</x:v>
+      </x:c>
+      <x:c r="G15" s="3" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="H15" s="3" t="str">
+        <x:v>DominicBytes</x:v>
+      </x:c>
+      <x:c r="I15" s="3" t="str">
+        <x:v>DECISIONS.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R423b50baed1a45e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33f1860a17334c3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2287,10 +2316,63 @@
         <x:v>High</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="3" t="str">
+        <x:v>SRC-019</x:v>
+      </x:c>
+      <x:c r="B21" s="3" t="str">
+        <x:v>v1.8.0 source baseline</x:v>
+      </x:c>
+      <x:c r="C21" s="3" t="str">
+        <x:v>https://github.com/limbonaut/limboai/releases/tag/v1.8.0</x:v>
+      </x:c>
+      <x:c r="D21" s="3" t="str">
+        <x:v>Release</x:v>
+      </x:c>
+      <x:c r="E21" s="3" t="str">
+        <x:v>LimboAI contributors</x:v>
+      </x:c>
+      <x:c r="F21" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="G21" s="3" t="str">
+        <x:v>Godot 4.6/4.7 upstream; Redot 26.2 target</x:v>
+      </x:c>
+      <x:c r="H21" s="3" t="str">
+        <x:v>C++ / SCons / GDExtension</x:v>
+      </x:c>
+      <x:c r="I21" s="3" t="str">
+        <x:v>MIT source; demo/logo separate</x:v>
+      </x:c>
+      <x:c r="J21" s="3" t="str">
+        <x:v>Selected complete-feature downstream baseline.</x:v>
+      </x:c>
+      <x:c r="K21" s="3" t="str">
+        <x:v>MS-005 to MS-055</x:v>
+      </x:c>
+      <x:c r="L21" s="3" t="str">
+        <x:v>Owner-authorized v1.8 baseline at commit 3fbd85118b924d50c10a495ad5c7175028649d77.</x:v>
+      </x:c>
+      <x:c r="M21" s="3" t="str">
+        <x:v>Requires compatibility adaptation for Redot's 4.5.2 API lineage.</x:v>
+      </x:c>
+      <x:c r="N21" s="3" t="str">
+        <x:v>Preserve the 1.8 public behavior/editor surface; adapt only proven engine-facing differences.</x:v>
+      </x:c>
+      <x:c r="O21" s="3" t="str">
+        <x:v>UPSTREAM_LOCK.md</x:v>
+      </x:c>
+      <x:c r="P21" s="3" t="str">
+        <x:v>Adapt</x:v>
+      </x:c>
+      <x:c r="Q21" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9d513f27bc84519"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94adadbcfcde4cfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2424,7 +2506,7 @@
         <x:v>Oracle build/run; hash and rights audits</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Complete</x:v>
+        <x:v>In progress: v1.8 baseline lock</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2453,7 +2535,7 @@
         <x:v>Fail-closed builds; bounded Redot runs</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Pending v1.8 build/load revalidation</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2482,7 +2564,7 @@
         <x:v>11-case fixture; GNT-01</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Automated complete; visible debugger blocked</x:v>
+        <x:v>Pending v1.8 vertical-slice revalidation</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2511,7 +2593,7 @@
         <x:v>11-case fixture; GNT-02</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Representative complete; coverage/perf blocked</x:v>
+        <x:v>Pending v1.8 feature/runtime revalidation</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2540,7 +2622,7 @@
         <x:v>Fixture plus visible protocol; GNT-03</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Automated complete; visible editor blocked</x:v>
+        <x:v>Pending v1.8 HSM/editor/migration revalidation</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2569,7 +2651,7 @@
         <x:v>Platform audits/CI; GNT-04</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Six binaries, deterministic archives, Windows/Linux headless clean installs, and Linux packed runtime complete; release gates blocked</x:v>
+        <x:v>Pending v1.8 desktop/package revalidation</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2581,7 +2663,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e7718a5bb8f4bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf41a9e7d8d444fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2954,10 +3036,37 @@
         <x:v>Provided binaries target Ubuntu 24.04/glibc 2.38+; older distributions require a source rebuild.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="72" customHeight="1">
+      <x:c r="A12" s="3" t="str">
+        <x:v>BLD-095</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="str">
+        <x:v>v1.8 scope amendment</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="str">
+        <x:v>Recorded the owner-authorized change from the v1.6 compatibility baseline to the complete upstream v1.8.0 feature baseline before modifying port source.</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>DECISIONS.md; docs/gamedev/implementation-plan.md; docs/gamedev/source-of-truth.xlsx</x:v>
+      </x:c>
+      <x:c r="F12" s="3"/>
+      <x:c r="G12" s="3" t="str">
+        <x:v>Clean branch; exact v1.8 tag and 48 non-merge commit delta verified</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I12" s="3" t="str">
+        <x:v>All implementation and release evidence is reopened for v1.8 revalidation.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red05e9cf6a0c4176"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16bacdd02bea4bbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3478,10 +3587,45 @@
         <x:v>Codex</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="60" customHeight="1">
+      <x:c r="A14" s="3" t="str">
+        <x:v>QA-115</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>Scope control</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>v1.8 baseline authorization and traceability</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="str">
+        <x:v>Clean port/redot-26.2 at 1229f9c; upstream v1.8.0 tag present</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>Scope change is recorded before source integration and prior 1.6 evidence remains historical</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="str">
+        <x:v>ADR-0010 and workbook rows identify v1.8.0@3fbd8511 and reopen affected gates</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="str">
+        <x:v>DECISIONS.md</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J14" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="K14" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dd999123d904150"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b6c388570a4f96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3617,25 +3761,25 @@
         <x:v>Baseline</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>4.5 versus current 4.6 API</x:v>
+        <x:v>Port complete LimboAI 1.8 behavior/editor surface onto Redot's 4.5.2 lineage</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
-        <x:v>Wrong baseline would prevent loading.</x:v>
+        <x:v>Godot 4.6/4.7 assumptions may break compilation, editor lifecycle, serialization, or runtime behavior.</x:v>
       </x:c>
       <x:c r="F3" s="3" t="str">
-        <x:v>Pinned verified v1.6.0; newest-vs-selected report retained.</x:v>
+        <x:v>Integrate v1.8 as one baseline, retain the locked Redot binding, and test each incompatibility at the narrow engine boundary.</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>Resolved</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Before MS-015 v1.8 revalidation</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>UPSTREAM_LOCK.md</x:v>
+        <x:v>DECISIONS.md</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3809,22 +3953,22 @@
         <x:v>Feature scope</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>Users may expect 1.7/1.8 features</x:v>
+        <x:v>Complete LimboAI 1.8 feature parity is now required</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
-        <x:v>Could create a misleading parity claim.</x:v>
+        <x:v>A partial backport would not satisfy the authorized product scope.</x:v>
       </x:c>
       <x:c r="F9" s="3" t="str">
-        <x:v>Version is 1.6.0+redot.26.2.1 and omissions/backport reports are explicit.</x:v>
+        <x:v>Merge the full v1.8 feature baseline, adapt 4.6/4.7 dependencies, and add direct feature regression coverage.</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>Mitigated</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>Before publication</x:v>
+        <x:v>Before source publication</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
         <x:v>reports/upstream-sync/v1.6.0-to-v1.8.0.md</x:v>
@@ -3841,22 +3985,22 @@
         <x:v>Publication</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str">
-        <x:v>Downstream repository/signing channel not authorized</x:v>
+        <x:v>Source publication is authorized; tag, release, and signing remain unauthorized</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
-        <x:v>Source and release cannot be published.</x:v>
+        <x:v>The source branch may be updated, but no release artifact or release claim may be published.</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
-        <x:v>Owner selects and authorizes repository, signing, tag, and release after gates pass.</x:v>
+        <x:v>Push only the verified source branch; request separate authorization for tags, releases, signing, or notarization.</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>DominicBytes</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Mitigated</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>Before publication</x:v>
+        <x:v>Before tag or release</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
         <x:v>BLOCKERS.md</x:v>
@@ -3897,7 +4041,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50b12436eade48d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re14386b4a6a243ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4085,7 +4229,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62e0d8a08984d60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbb551f6ae6b4d9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4257,7 +4401,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57731cb8c4d14210"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eced115e7c34d5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record validated LimboAI 1.8 Redot port
</commit_message>
<xml_diff>
--- a/docs/gamedev/source-of-truth.xlsx
+++ b/docs/gamedev/source-of-truth.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R640a302ed2c444e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="Red8624fc5cd44913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R35fa68da42894afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="R1734571317c54430"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R2776dec544584180"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Rf8f1f53615a2437a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="Re600bc6666e441bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rf3bb6f2bb0464d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="Rc9cfedd505e04386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra8228d0795fc4331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R23e2322f45044f8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Ra17b4a5fda754062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rdff6086b89d64ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R0f99f9520dfd4afa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="R3c33963c5f944cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R0f5ba5f0c35b4672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="R0f4eb6a5d5a345cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R32a9bcb70dab4e31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -213,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I12" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I12"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I15" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I15"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K14" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:K14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K15" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:K15"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -270,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="GameDev8" displayName="GameDev8" ref="A1:L3" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:L3"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="GameDev8" displayName="GameDev8" ref="A1:L11" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:L11"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -640,13 +640,13 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>LimboAI v1.8.0 Redot port in progress; the verified 1.6 implementation is retained as a checkpoint and all implementation gates are reopened for the new baseline</x:v>
+        <x:v>LimboAI v1.8.0 Redot port complete locally; source publication authorized, while visible-editor, native macOS runtime, and binary-release gates remain open</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>Owner-authorized scope expansion to the complete v1.8 feature set on Redot 26.2</x:v>
+        <x:v>Exact v1.8 tag merged at a6c0d08; six desktop binaries, 13-case fixtures, demo, deterministic packages, and rights audits pass</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -680,7 +680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a3aa6dd9d5742d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3acf99dad94466e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -901,7 +901,7 @@
         <x:v>Port current master directly; lock v1.6.0 without build proof</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>Codex</x:v>
@@ -1075,7 +1075,7 @@
         <x:v>Bulk merge newer releases</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
         <x:v>Codex</x:v>
@@ -1104,7 +1104,7 @@
         <x:v>Keep the patch solely because it is newer</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Accepted</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
         <x:v>Codex</x:v>
@@ -1174,7 +1174,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33f1860a17334c3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7008a49f77204622"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1434,7 +1434,7 @@
         <x:v>SRC-002</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>v1.6.0 source baseline</x:v>
+        <x:v>v1.6.0 compatibility checkpoint</x:v>
       </x:c>
       <x:c r="C4" s="3" t="str">
         <x:v>https://github.com/limbonaut/limboai/releases/tag/v1.6.0</x:v>
@@ -1458,25 +1458,25 @@
         <x:v>MIT source; demo/logo separate</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Selected downstream source baseline.</x:v>
+        <x:v>Historical API-lineage and regression checkpoint.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
         <x:v>MS-005</x:v>
       </x:c>
       <x:c r="L4" s="3" t="str">
-        <x:v>Verified tag commit 91b22a187f7cd701e25eedd6dcff34179795e687.</x:v>
+        <x:v>Verified former baseline retained as compatibility evidence.</x:v>
       </x:c>
       <x:c r="M4" s="3" t="str">
         <x:v>Builds under Godot 4.5.2 and Redot 26.2.</x:v>
       </x:c>
       <x:c r="N4" s="3" t="str">
-        <x:v>Retain public names; apply only verified isolated fixes.</x:v>
+        <x:v>Retain evidence; do not describe as the selected feature baseline.</x:v>
       </x:c>
       <x:c r="O4" s="3" t="str">
         <x:v>UPSTREAM_LOCK.md</x:v>
       </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>Adopt</x:v>
+        <x:v>Historical</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="str">
         <x:v>High</x:v>
@@ -1952,7 +1952,7 @@
         <x:v>SRC-012</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>LimboAI v1.8.0 comparison</x:v>
+        <x:v>v1.8.0 preflight snapshot</x:v>
       </x:c>
       <x:c r="C14" s="3" t="str">
         <x:v>https://github.com/limbonaut/limboai/commit/3fbd85118b924d50c10a495ad5c7175028649d77</x:v>
@@ -1976,25 +1976,25 @@
         <x:v>MIT source; demo/logo separate</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
-        <x:v>Newest-versus-selected comparison.</x:v>
+        <x:v>Historical preflight comparison; exact tag is now SRC-019.</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
         <x:v>MS-005</x:v>
       </x:c>
       <x:c r="L14" s="3" t="str">
-        <x:v>Newest checked stable source requires Godot 4.6 APIs.</x:v>
+        <x:v>Preflight identified the later feature/API delta.</x:v>
       </x:c>
       <x:c r="M14" s="3" t="str">
-        <x:v>Not compatible with the Redot 26.2 / Godot 4.5 lineage.</x:v>
+        <x:v>Requires Redot 4.5-lineage compatibility work.</x:v>
       </x:c>
       <x:c r="N14" s="3" t="str">
-        <x:v>Retain only as comparison; backport isolated verified fixes.</x:v>
+        <x:v>Use SRC-019 and UPSTREAM_LOCK.md for the selected baseline.</x:v>
       </x:c>
       <x:c r="O14" s="3" t="str">
-        <x:v>reports/api-diffs/limboai-newest-vs-selected.md</x:v>
+        <x:v>docs/gamedev/preflight-report.md</x:v>
       </x:c>
       <x:c r="P14" s="3" t="str">
-        <x:v>Adapt</x:v>
+        <x:v>Historical</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="str">
         <x:v>High</x:v>
@@ -2162,7 +2162,7 @@
         <x:v>SRC-016</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
-        <x:v>Selected source commit</x:v>
+        <x:v>v1.6 compatibility-checkpoint commit</x:v>
       </x:c>
       <x:c r="C18" s="3" t="str">
         <x:v>https://github.com/limbonaut/limboai/commit/91b22a187f7cd701e25eedd6dcff34179795e687</x:v>
@@ -2186,25 +2186,25 @@
         <x:v>MIT</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Immutable upstream baseline.</x:v>
+        <x:v>Historical compatibility checkpoint.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>MS-005</x:v>
       </x:c>
       <x:c r="L18" s="3" t="str">
-        <x:v>Full-history tag resolution for v1.6.0.</x:v>
+        <x:v>Immutable former baseline used for the 1.6-to-1.8 range.</x:v>
       </x:c>
       <x:c r="M18" s="3" t="str">
-        <x:v>Oracle and Redot builds pass.</x:v>
+        <x:v>Oracle and Redot builds passed at the checkpoint.</x:v>
       </x:c>
       <x:c r="N18" s="3" t="str">
-        <x:v>Never replace with mutable master.</x:v>
+        <x:v>Retain for provenance and regression history.</x:v>
       </x:c>
       <x:c r="O18" s="3" t="str">
         <x:v>UPSTREAM_LOCK.md</x:v>
       </x:c>
       <x:c r="P18" s="3" t="str">
-        <x:v>Adopt</x:v>
+        <x:v>Historical</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="str">
         <x:v>High</x:v>
@@ -2372,7 +2372,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94adadbcfcde4cfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3110d63b25eb44c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2506,7 +2506,7 @@
         <x:v>Oracle build/run; hash and rights audits</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>In progress: v1.8 baseline lock</x:v>
+        <x:v>Complete: exact v1.8 baseline and rights lock</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2535,7 +2535,7 @@
         <x:v>Fail-closed builds; bounded Redot runs</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Pending v1.8 build/load revalidation</x:v>
+        <x:v>Complete locally: Windows/Linux load; macOS structural</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2561,10 +2561,10 @@
         <x:v>Tree/resource/blackboard/BTPlayer parity plus visible debugger</x:v>
       </x:c>
       <x:c r="F5" s="3" t="str">
-        <x:v>11-case fixture; GNT-01</x:v>
+        <x:v>13-case fixture; GNT-01</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Pending v1.8 vertical-slice revalidation</x:v>
+        <x:v>Automated PASS; visible debugger gate open</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2590,10 +2590,10 @@
         <x:v>Representative tasks, blackboards, multi-agent, custom tasks, runtime view</x:v>
       </x:c>
       <x:c r="F6" s="3" t="str">
-        <x:v>11-case fixture; GNT-02</x:v>
+        <x:v>13-case fixture; GNT-02</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Pending v1.8 feature/runtime revalidation</x:v>
+        <x:v>Representative runtime PASS; full/performance gates open</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2622,7 +2622,7 @@
         <x:v>Fixture plus visible protocol; GNT-03</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Pending v1.8 HSM/editor/migration revalidation</x:v>
+        <x:v>HSM cargo/runtime PASS; visible editor gate open</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2651,7 +2651,7 @@
         <x:v>Platform audits/CI; GNT-04</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Pending v1.8 desktop/package revalidation</x:v>
+        <x:v>Local package PASS; native macOS and binary-release gates open</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
         <x:v>Codex</x:v>
@@ -2663,7 +2663,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf41a9e7d8d444fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R685b99bc61f547cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3054,19 +3054,106 @@
       </x:c>
       <x:c r="F12" s="3"/>
       <x:c r="G12" s="3" t="str">
-        <x:v>Clean branch; exact v1.8 tag and 48 non-merge commit delta verified</x:v>
+        <x:v>Clean branch; exact v1.8 tag and 49 non-merge commit delta verified</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
         <x:v>All implementation and release evidence is reopened for v1.8 revalidation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="72" customHeight="1">
+      <x:c r="A13" s="3" t="str">
+        <x:v>BLD-105</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="str">
+        <x:v>v1.8 source integration</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="str">
+        <x:v>Merged exact upstream v1.8.0 as a second parent and retained only documented Redot engine/build/test adaptations.</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="str">
+        <x:v>C++ source; demo; reports/api-diffs; reports/upstream-sync</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:v>a6c0d0863fb98f93d1219acbe6fc07b3608614be</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="str">
+        <x:v>49 non-merge commits accounted for; Python tests PASS; Redot demo PASS</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I13" s="3" t="str">
+        <x:v>Includes task palette/favorites, probability/status UI, runtime blackboard inspection, HSM cargo, and 1.8 safety fixes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="72" customHeight="1">
+      <x:c r="A14" s="3" t="str">
+        <x:v>BLD-115</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>v1.8 desktop validation</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>Rebuilt and audited Windows/Linux editor and release libraries plus macOS universal frameworks from the committed port.</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="str">
+        <x:v>external platform projects; reports/test-results/automated-desktop.md</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>a6c0d0863fb98f93d1219acbe6fc07b3608614be</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="str">
+        <x:v>PE/ELF/Mach-O audits; four direct 13-case runtime profiles</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>Native macOS runtime remains a hosted gate; Zig libc++ diagnostics are toolchain-only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="3" t="str">
+        <x:v>BLD-125</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C15" s="3" t="str">
+        <x:v>v1.8 clean package</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="str">
+        <x:v>Produced byte-identical core/demo archives twice, extracted core, ran four 13-case profiles, and passed an 89-file packed Linux release run.</x:v>
+      </x:c>
+      <x:c r="E15" s="3" t="str">
+        <x:v>scripts/package_release.py; final archive extraction; release-manifest.json</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="str">
+        <x:v>a6c0d0863fb98f93d1219acbe6fc07b3608614be</x:v>
+      </x:c>
+      <x:c r="G15" s="3" t="str">
+        <x:v>Core D4C33970...; demo 7F4C8A31...; packed PCK 1B453F33...</x:v>
+      </x:c>
+      <x:c r="H15" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I15" s="3" t="str">
+        <x:v>Core 78 entries; demo 171 entries; source push authorized without tag or release.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16bacdd02bea4bbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4db6ea95ee9044d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3222,7 +3309,7 @@
         <x:v>Bounded fixture passes with no unexplained errors</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Windows/Linux editor and forced-release fixtures pass all 11 cases</x:v>
+        <x:v>Windows/Linux editor and forced-release fixtures pass all 13 cases</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3318,16 +3405,16 @@
         <x:v>MS-025 to MS-045</x:v>
       </x:c>
       <x:c r="D6" s="3" t="str">
-        <x:v>Windows editor/release fixture</x:v>
+        <x:v>Windows editor/release v1.8 fixture</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
-        <x:v>Redot 26.2 Windows x86-64</x:v>
+        <x:v>Redot 26.2 Windows x86-64; committed port</x:v>
       </x:c>
       <x:c r="F6" s="3" t="str">
-        <x:v>11 cases and zero suspicious lines</x:v>
+        <x:v>13 cases and zero suspicious lines</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Both profiles pass; release SHA E01C5F14...</x:v>
+        <x:v>Both final and archive profiles pass; release SHA 312A6EB5...</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3353,16 +3440,16 @@
         <x:v>MS-025 to MS-045</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>Linux editor/release fixture</x:v>
+        <x:v>Linux editor/release v1.8 fixture</x:v>
       </x:c>
       <x:c r="E7" s="3" t="str">
-        <x:v>Redot 26.2 Linux x86-64</x:v>
+        <x:v>Redot 26.2 Ubuntu 24.04 x86-64; committed port</x:v>
       </x:c>
       <x:c r="F7" s="3" t="str">
-        <x:v>11 cases and zero suspicious lines</x:v>
+        <x:v>13 cases and zero suspicious lines</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Both profiles pass; release SHA 2291FCAB...</x:v>
+        <x:v>Both final and archive profiles pass; release SHA 873BD867...</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3394,10 +3481,10 @@
         <x:v>Pinned Zig cross-build; x86-64 + arm64</x:v>
       </x:c>
       <x:c r="F8" s="3" t="str">
-        <x:v>Two slices, 11.0, system dependency, stable ID, export, no leaks</x:v>
+        <x:v>Two slices, macOS 11.0, system dependency, stable ID, export, no leaks</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Both editor/release frameworks pass strict parser</x:v>
+        <x:v>Editor 3C45D891... and release 19640178... pass strict parser</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3461,13 +3548,13 @@
         <x:v>Deterministic archive comparison</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
-        <x:v>Clean source commit f51be6ba; two independent output roots</x:v>
+        <x:v>Clean source commit a6c0d08; two independent output roots</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
         <x:v>Core and demo ZIP bytes match</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Core FF4E028C...D1FEE70 and demo 30456BCF...ECC8A3 match exactly</x:v>
+        <x:v>Core D4C33970...8C39075 and demo 7F4C8A31...6F3DE3 match exactly</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
         <x:v>reports/licenses/limboai-package-audit.md</x:v>
@@ -3499,10 +3586,10 @@
         <x:v>Windows host and offline Ubuntu 24.04; editor and template_release</x:v>
       </x:c>
       <x:c r="F11" s="3" t="str">
-        <x:v>All 11 cases pass with zero suspicious lines</x:v>
+        <x:v>All 13 cases pass with zero suspicious lines</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Four profiles pass from a fresh archive extraction</x:v>
+        <x:v>Four profiles pass from a fresh 1.8 archive extraction</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3534,10 +3621,10 @@
         <x:v>Exact packaged Linux template_release library; 89-file PCK</x:v>
       </x:c>
       <x:c r="F12" s="3" t="str">
-        <x:v>All 11 cases pass with zero suspicious lines</x:v>
+        <x:v>All 13 cases pass</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>PCK SHA-256 63F19B07...645AD13CB; runtime PASS</x:v>
+        <x:v>PCK SHA-256 1B453F33...B1D293E; runtime PASS</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
         <x:v>reports/test-results/automated-desktop.md</x:v>
@@ -3601,13 +3688,13 @@
         <x:v>v1.8 baseline authorization and traceability</x:v>
       </x:c>
       <x:c r="E14" s="3" t="str">
-        <x:v>Clean port/redot-26.2 at 1229f9c; upstream v1.8.0 tag present</x:v>
+        <x:v>Clean merge commit a6c0d08; upstream v1.8.0 second parent</x:v>
       </x:c>
       <x:c r="F14" s="3" t="str">
-        <x:v>Scope change is recorded before source integration and prior 1.6 evidence remains historical</x:v>
+        <x:v>Every 1.6-to-1.8 commit is adopted or a downstream delta is documented</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>ADR-0010 and workbook rows identify v1.8.0@3fbd8511 and reopen affected gates</x:v>
+        <x:v>49 non-merge commits present; narrow Redot delta report complete</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
         <x:v>DECISIONS.md</x:v>
@@ -3619,13 +3706,48 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="3" t="str">
+        <x:v>QA-125</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C15" s="3" t="str">
+        <x:v>v1.8 feature retention</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="str">
+        <x:v>Runtime inspection, HSM cargo, modern palette/favorites, probability/status, debugger and safety changes</x:v>
+      </x:c>
+      <x:c r="E15" s="3" t="str">
+        <x:v>Exact v1.8 source plus committed Redot build</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="str">
+        <x:v>All source present; direct runtime cases pass; editor initializes</x:v>
+      </x:c>
+      <x:c r="G15" s="3" t="str">
+        <x:v>Blackboard inspection and cargo cases PASS; final demo exits cleanly</x:v>
+      </x:c>
+      <x:c r="H15" s="3" t="str">
+        <x:v>reports/api-diffs/limboai-newest-vs-selected.md</x:v>
+      </x:c>
+      <x:c r="I15" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J15" s="3" t="str">
+        <x:v>PASS (visible UX gated)</x:v>
+      </x:c>
+      <x:c r="K15" s="3" t="str">
         <x:v>Codex</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87b6c388570a4f96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1051286997b24e58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3761,25 +3883,25 @@
         <x:v>Baseline</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
-        <x:v>Port complete LimboAI 1.8 behavior/editor surface onto Redot's 4.5.2 lineage</x:v>
+        <x:v>Complete LimboAI 1.8 behavior/editor surface on Redot's 4.5.2 lineage</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
-        <x:v>Godot 4.6/4.7 assumptions may break compilation, editor lifecycle, serialization, or runtime behavior.</x:v>
+        <x:v>Godot 4.6/4.7 assumptions could break compilation, editor lifecycle, serialization, or runtime behavior.</x:v>
       </x:c>
       <x:c r="F3" s="3" t="str">
-        <x:v>Integrate v1.8 as one baseline, retain the locked Redot binding, and test each incompatibility at the narrow engine boundary.</x:v>
+        <x:v>Exact-tag merge, narrow Redot adaptations, six builds, demo run, and 13-case runtime validation.</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Mitigated locally</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Before MS-015 v1.8 revalidation</x:v>
+        <x:v>Visible editor and native macOS before release claim</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>DECISIONS.md</x:v>
+        <x:v>reports/api-diffs/limboai-newest-vs-selected.md</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -3895,7 +4017,7 @@
         <x:v>Some task families or malformed inputs may remain untested.</x:v>
       </x:c>
       <x:c r="F7" s="3" t="str">
-        <x:v>Representative 11-case fixture passes; full 53-test mapping remains a GNT-02 blocker.</x:v>
+        <x:v>Representative 13-case fixture passes; full upstream-test and malformed-input mapping remains a GNT-02 blocker.</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
         <x:v>Codex</x:v>
@@ -3953,22 +4075,22 @@
         <x:v>Feature scope</x:v>
       </x:c>
       <x:c r="D9" s="3" t="str">
-        <x:v>Complete LimboAI 1.8 feature parity is now required</x:v>
+        <x:v>Complete LimboAI 1.8 feature parity is required</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
         <x:v>A partial backport would not satisfy the authorized product scope.</x:v>
       </x:c>
       <x:c r="F9" s="3" t="str">
-        <x:v>Merge the full v1.8 feature baseline, adapt 4.6/4.7 dependencies, and add direct feature regression coverage.</x:v>
+        <x:v>Merged exact v1.8 tag and verified the previously omitted feature groups directly.</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>Before source publication</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
         <x:v>reports/upstream-sync/v1.6.0-to-v1.8.0.md</x:v>
@@ -3988,10 +4110,10 @@
         <x:v>Source publication is authorized; tag, release, and signing remain unauthorized</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
-        <x:v>The source branch may be updated, but no release artifact or release claim may be published.</x:v>
+        <x:v>The verified source may be pushed, but binary release objects still require separate authority.</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
-        <x:v>Push only the verified source branch; request separate authorization for tags, releases, signing, or notarization.</x:v>
+        <x:v>Push only port/redot-26.2 to dominicbytes/redot-limbo; create no tag, release, signature, or notarization.</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>DominicBytes</x:v>
@@ -4041,7 +4163,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re14386b4a6a243ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re592db03018c412c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4188,7 +4310,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="3" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="3" ht="78" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="str">
         <x:v>REL-001</x:v>
       </x:c>
@@ -4220,16 +4342,320 @@
         <x:v>No publication</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="L3" s="3" t="str">
-        <x:v>Linux requires glibc 2.38+; native macOS, visible editor, controlled performance, native Windows/macOS export, signing, and owner authorization gates remain.</x:v>
+        <x:v>Historical 1.6 package evidence; replaced by the verified v1.8 rows below.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="78" customHeight="1">
+      <x:c r="A4" s="3" t="str">
+        <x:v>REL-010</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C4" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E4" s="3" t="str">
+        <x:v>Windows x86-64</x:v>
+      </x:c>
+      <x:c r="F4" s="3" t="str">
+        <x:v>editor</x:v>
+      </x:c>
+      <x:c r="G4" s="3" t="str">
+        <x:v>liblimboai.windows.editor.x86_64.dll</x:v>
+      </x:c>
+      <x:c r="H4" s="3" t="str">
+        <x:v>ECFA90017DE6BEF0945C5FEA05CC8368F5F4BA6CBBC4B09347AD2ED3C90F914E</x:v>
+      </x:c>
+      <x:c r="I4" s="3" t="str">
+        <x:v>PE audit; 13-case direct/archive</x:v>
+      </x:c>
+      <x:c r="J4" s="3" t="str">
+        <x:v>Core archive</x:v>
+      </x:c>
+      <x:c r="K4" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="L4" s="3" t="str">
+        <x:v>Not signed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="78" customHeight="1">
+      <x:c r="A5" s="3" t="str">
+        <x:v>REL-020</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C5" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D5" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E5" s="3" t="str">
+        <x:v>Windows x86-64</x:v>
+      </x:c>
+      <x:c r="F5" s="3" t="str">
+        <x:v>template_release</x:v>
+      </x:c>
+      <x:c r="G5" s="3" t="str">
+        <x:v>liblimboai.windows.template_release.x86_64.dll</x:v>
+      </x:c>
+      <x:c r="H5" s="3" t="str">
+        <x:v>312A6EB51B83A7EE79CF705F650EB40E2955C1820FD7F2A21F34413A0DC85E6B</x:v>
+      </x:c>
+      <x:c r="I5" s="3" t="str">
+        <x:v>PE audit; forced 13-case direct/archive</x:v>
+      </x:c>
+      <x:c r="J5" s="3" t="str">
+        <x:v>Core archive</x:v>
+      </x:c>
+      <x:c r="K5" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="L5" s="3" t="str">
+        <x:v>Not signed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="78" customHeight="1">
+      <x:c r="A6" s="3" t="str">
+        <x:v>REL-030</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="str">
+        <x:v>Linux x86-64</x:v>
+      </x:c>
+      <x:c r="F6" s="3" t="str">
+        <x:v>editor</x:v>
+      </x:c>
+      <x:c r="G6" s="3" t="str">
+        <x:v>liblimboai.linux.editor.x86_64.so</x:v>
+      </x:c>
+      <x:c r="H6" s="3" t="str">
+        <x:v>FCDB32CF5A250F72077A980DAE9B0BAE8C5FEF60C04D8797439EDC4FA0BAA405</x:v>
+      </x:c>
+      <x:c r="I6" s="3" t="str">
+        <x:v>ELF/glibc audit; 13-case direct/archive</x:v>
+      </x:c>
+      <x:c r="J6" s="3" t="str">
+        <x:v>Core archive</x:v>
+      </x:c>
+      <x:c r="K6" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="L6" s="3" t="str">
+        <x:v>glibc 2.38 floor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="78" customHeight="1">
+      <x:c r="A7" s="3" t="str">
+        <x:v>REL-040</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="str">
+        <x:v>Linux x86-64</x:v>
+      </x:c>
+      <x:c r="F7" s="3" t="str">
+        <x:v>template_release</x:v>
+      </x:c>
+      <x:c r="G7" s="3" t="str">
+        <x:v>liblimboai.linux.template_release.x86_64.so</x:v>
+      </x:c>
+      <x:c r="H7" s="3" t="str">
+        <x:v>873BD867F3A844C65020F6F278A85A8F2B273A3FCAAB9EA5D2D3E629ABFE9656</x:v>
+      </x:c>
+      <x:c r="I7" s="3" t="str">
+        <x:v>ELF/glibc audit; forced 13-case; packed PCK</x:v>
+      </x:c>
+      <x:c r="J7" s="3" t="str">
+        <x:v>Core archive</x:v>
+      </x:c>
+      <x:c r="K7" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="L7" s="3" t="str">
+        <x:v>glibc 2.38 floor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="78" customHeight="1">
+      <x:c r="A8" s="3" t="str">
+        <x:v>REL-050</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>macOS universal</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>editor</x:v>
+      </x:c>
+      <x:c r="G8" s="3" t="str">
+        <x:v>liblimboai.macos.editor.framework</x:v>
+      </x:c>
+      <x:c r="H8" s="3" t="str">
+        <x:v>3C45D891428A469CA6DF2C54433E073C3BB17A0913630F40F175BD385F42520C</x:v>
+      </x:c>
+      <x:c r="I8" s="3" t="str">
+        <x:v>Mach-O structural audit</x:v>
+      </x:c>
+      <x:c r="J8" s="3" t="str">
+        <x:v>Core archive</x:v>
+      </x:c>
+      <x:c r="K8" s="3" t="str">
+        <x:v>PASS (structural)</x:v>
+      </x:c>
+      <x:c r="L8" s="3" t="str">
+        <x:v>Native runtime gated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="78" customHeight="1">
+      <x:c r="A9" s="3" t="str">
+        <x:v>REL-060</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="str">
+        <x:v>macOS universal</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="str">
+        <x:v>template_release</x:v>
+      </x:c>
+      <x:c r="G9" s="3" t="str">
+        <x:v>liblimboai.macos.template_release.framework</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="str">
+        <x:v>19640178510822407C268CAFF28F91DEFCAC0DFB3A88179BD85859D9925A5FA3</x:v>
+      </x:c>
+      <x:c r="I9" s="3" t="str">
+        <x:v>Mach-O structural audit</x:v>
+      </x:c>
+      <x:c r="J9" s="3" t="str">
+        <x:v>Core archive</x:v>
+      </x:c>
+      <x:c r="K9" s="3" t="str">
+        <x:v>PASS (structural)</x:v>
+      </x:c>
+      <x:c r="L9" s="3" t="str">
+        <x:v>Native runtime gated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="78" customHeight="1">
+      <x:c r="A10" s="3" t="str">
+        <x:v>REL-070</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>Desktop core</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>deterministic ZIP</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>redot-limboai-1.8.0+redot.26.2.1-core.zip</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>D4C339702D7F3DCCDF5D414EDE7EA1F5C0174385DB65F7A75685CFCA88C39075</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="str">
+        <x:v>78 entries; byte-identical; clean installs</x:v>
+      </x:c>
+      <x:c r="J10" s="3" t="str">
+        <x:v>Local dist only</x:v>
+      </x:c>
+      <x:c r="K10" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="L10" s="3" t="str">
+        <x:v>No public release created</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="78" customHeight="1">
+      <x:c r="A11" s="3" t="str">
+        <x:v>REL-080</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="str">
+        <x:v>1.8.0+redot.26.2.1</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="str">
+        <x:v>a6c0d08</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="str">
+        <x:v>Demo/tutorial</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="str">
+        <x:v>deterministic ZIP</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="str">
+        <x:v>redot-limboai-1.8.0+redot.26.2.1-demo.zip</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
+        <x:v>7F4C8A31C51BE566357E2D37966166730C1B5697CA8350F0D18FACEC426F3DE3</x:v>
+      </x:c>
+      <x:c r="I11" s="3" t="str">
+        <x:v>171 entries; byte-identical; rights inventory</x:v>
+      </x:c>
+      <x:c r="J11" s="3" t="str">
+        <x:v>Local dist only</x:v>
+      </x:c>
+      <x:c r="K11" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="L11" s="3" t="str">
+        <x:v>CC BY 4.0 and OFL notices included</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbb551f6ae6b4d9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d5156e709ba4457"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4401,7 +4827,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eced115e7c34d5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ebf8257ce254328"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize Redot port publication record
</commit_message>
<xml_diff>
--- a/docs/gamedev/source-of-truth.xlsx
+++ b/docs/gamedev/source-of-truth.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra8228d0795fc4331"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R23e2322f45044f8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="Ra17b4a5fda754062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rdff6086b89d64ee8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R0f99f9520dfd4afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="R3c33963c5f944cae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R0f5ba5f0c35b4672"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="R0f4eb6a5d5a345cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R32a9bcb70dab4e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd9328df6d95a4cec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R1316681a7e6348a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R05a30e8eb0954b3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="R6180d29bddde4dee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R4f326512c650450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Red964becacee4134"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="Rd49afbf8b2794a6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="R02f897f101a34189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R37b37d1fb7b24b63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -213,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I15" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I15"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I16" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I16"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -640,13 +640,13 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>LimboAI v1.8.0 Redot port complete locally; source publication authorized, while visible-editor, native macOS runtime, and binary-release gates remain open</x:v>
+        <x:v>LimboAI v1.8.0 Redot port implemented, validated, and published to the redot-limbo source fork; visible-editor, native macOS runtime, and binary-release gates remain open</x:v>
       </x:c>
       <x:c r="C7" s="3" t="str">
         <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D7" s="3" t="str">
-        <x:v>Exact v1.8 tag merged at a6c0d08; six desktop binaries, 13-case fixtures, demo, deterministic packages, and rights audits pass</x:v>
+        <x:v>Default branch port/redot-26.2 published to dominicbytes/redot-limbo; repository description identifies the Redot 26.2 port; no tag or release created</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -680,7 +680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3acf99dad94466e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29c899037897417b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1174,7 +1174,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7008a49f77204622"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re43bc6176d5e4e85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2372,7 +2372,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3110d63b25eb44c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0aa7f104d4c446a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2663,7 +2663,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R685b99bc61f547cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64794698fe2e4fee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3150,10 +3150,39 @@
         <x:v>Core 78 entries; demo 171 entries; source push authorized without tag or release.</x:v>
       </x:c>
     </x:row>
+    <x:row r="16" ht="72" customHeight="1">
+      <x:c r="A16" s="3" t="str">
+        <x:v>BLD-135</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C16" s="3" t="str">
+        <x:v>Source publication</x:v>
+      </x:c>
+      <x:c r="D16" s="3" t="str">
+        <x:v>Published the verified v1.8 Redot source branch and updated the fork description while preserving the owner's intervening README commit.</x:v>
+      </x:c>
+      <x:c r="E16" s="3" t="str">
+        <x:v>https://github.com/dominicbytes/redot-limbo/tree/port/redot-26.2</x:v>
+      </x:c>
+      <x:c r="F16" s="3" t="str">
+        <x:v>54d383d</x:v>
+      </x:c>
+      <x:c r="G16" s="3" t="str">
+        <x:v>Remote default branch and description verified; no tag or GitHub release created</x:v>
+      </x:c>
+      <x:c r="H16" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I16" s="3" t="str">
+        <x:v>Binary-release, signing, notarization, visible-editor, and native macOS gates remain open.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4db6ea95ee9044d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7d74da033644bc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3747,7 +3776,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1051286997b24e58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8664e637510f420f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4107,19 +4136,19 @@
         <x:v>Publication</x:v>
       </x:c>
       <x:c r="D10" s="3" t="str">
-        <x:v>Source publication is authorized; tag, release, and signing remain unauthorized</x:v>
+        <x:v>Source publication is complete; tag, release, and signing remain unauthorized</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
-        <x:v>The verified source may be pushed, but binary release objects still require separate authority.</x:v>
+        <x:v>The verified source branch is public, but binary release objects still require separate authority.</x:v>
       </x:c>
       <x:c r="F10" s="3" t="str">
-        <x:v>Push only port/redot-26.2 to dominicbytes/redot-limbo; create no tag, release, signature, or notarization.</x:v>
+        <x:v>Keep port/redot-26.2 as the source branch; request separate authorization for tags, releases, signing, or notarization.</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
         <x:v>DominicBytes</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Mitigated</x:v>
+        <x:v>Resolved for source</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
         <x:v>Before tag or release</x:v>
@@ -4163,7 +4192,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re592db03018c412c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R233d3a632004447c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4655,7 +4684,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d5156e709ba4457"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02ffc1c38df74b00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4827,7 +4856,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ebf8257ce254328"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c4dd1c488244708"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>